<commit_message>
Har tilføjet scripts til at generere sandsynligheder og optimal policy
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,41 +459,6 @@
           <t>demand_5</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>demand_6</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>demand_7</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>demand_8</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>demand_9</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>demand_10</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>demand_11</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>demand_12</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -502,43 +467,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.00250082819635074</v>
+        <v>0.085685596340511</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01500496917810444</v>
+        <v>0.2142139908512775</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04501490753431331</v>
+        <v>0.2677674885640969</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09002981506862662</v>
+        <v>0.223139573803414</v>
       </c>
       <c r="F2" t="n">
-        <v>0.13504472260294</v>
+        <v>0.1394622336271338</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1620536671235279</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.1620536671235279</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.1389031432487382</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.1041773574365537</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.06945157162436912</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.04167094297462147</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.02272960525888443</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.01136480262944222</v>
+        <v>0.06973111681356689</v>
       </c>
     </row>
     <row r="3">
@@ -548,43 +492,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001527926727909667</v>
+        <v>0.03521094473532189</v>
       </c>
       <c r="C3" t="n">
-        <v>0.009931523731412832</v>
+        <v>0.1232383065736266</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03227745212709171</v>
+        <v>0.2156670365038466</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06993447960869871</v>
+        <v>0.251611542587821</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1136435293641354</v>
+        <v>0.2201600997643434</v>
       </c>
       <c r="G3" t="n">
-        <v>0.147736588173376</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.1600479705211574</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.148615972626789</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.120750477759266</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.08720867838169212</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.05668564094809989</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.03349606056024084</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.01814369947013045</v>
+        <v>0.1541120698350404</v>
       </c>
     </row>
     <row r="4">
@@ -594,43 +517,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0009371857689742059</v>
+        <v>0.02332814930015552</v>
       </c>
       <c r="C4" t="n">
-        <v>0.006560300382819442</v>
+        <v>0.0933125972006221</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02296105133986804</v>
+        <v>0.1866251944012442</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0535757864596921</v>
+        <v>0.2488335925349922</v>
       </c>
       <c r="F4" t="n">
-        <v>0.09375762630446119</v>
+        <v>0.2488335925349922</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1312606768262456</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1531374562972866</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1531374562972866</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.1339952742601258</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.1042185466467645</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.07295298265273516</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.04642462532446782</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.02708103143927289</v>
+        <v>0.1990668740279938</v>
       </c>
     </row>
     <row r="5">
@@ -640,43 +542,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0005777338876722062</v>
+        <v>0.03521094473532189</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004333004157541547</v>
+        <v>0.1232383065736266</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0162487655907808</v>
+        <v>0.2156670365038466</v>
       </c>
       <c r="E5" t="n">
-        <v>0.040621913976952</v>
+        <v>0.251611542587821</v>
       </c>
       <c r="F5" t="n">
-        <v>0.076166088706785</v>
+        <v>0.2201600997643434</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1142491330601775</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.1428114163252219</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.1530122317770234</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.1434489672909595</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.1195408060757996</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.08965560455684968</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.06112882128876114</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.03820551330547572</v>
+        <v>0.1541120698350404</v>
       </c>
     </row>
     <row r="6">
@@ -686,43 +567,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0002238171714130312</v>
+        <v>0.05434782608695652</v>
       </c>
       <c r="C6" t="n">
-        <v>0.001902445957010766</v>
+        <v>0.1630434782608696</v>
       </c>
       <c r="D6" t="n">
-        <v>0.008085395317295754</v>
+        <v>0.2445652173913044</v>
       </c>
       <c r="E6" t="n">
-        <v>0.02290862006567131</v>
+        <v>0.2445652173913044</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04868081763955152</v>
+        <v>0.1834239130434783</v>
       </c>
       <c r="G6" t="n">
-        <v>0.08275738998723758</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.1172396358152533</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.1423624149185218</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.1512600658509294</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1428567288592111</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.1214282195303294</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.09383089690980004</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.06646355197777501</v>
+        <v>0.1100543478260869</v>
       </c>
     </row>
     <row r="7">
@@ -732,43 +592,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.006751577432172175</v>
+        <v>0.1376146788990826</v>
       </c>
       <c r="C7" t="n">
-        <v>0.03375788716086087</v>
+        <v>0.2752293577981652</v>
       </c>
       <c r="D7" t="n">
-        <v>0.08439471790215218</v>
+        <v>0.2752293577981652</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1406578631702536</v>
+        <v>0.1834862385321101</v>
       </c>
       <c r="F7" t="n">
-        <v>0.175822328962817</v>
+        <v>0.09174311926605505</v>
       </c>
       <c r="G7" t="n">
-        <v>0.175822328962817</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.1465186074690142</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.104656148192153</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.06541009262009563</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.03633894034449758</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.01816947017224878</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.008258850078294903</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.003441187532622876</v>
+        <v>0.03669724770642202</v>
       </c>
     </row>
     <row r="8">
@@ -778,43 +617,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.01111794801934412</v>
+        <v>0.224128874102609</v>
       </c>
       <c r="C8" t="n">
-        <v>0.05003076608704855</v>
+        <v>0.3361933111539135</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1125692236958593</v>
+        <v>0.2521449833654351</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1688538355437889</v>
+        <v>0.1260724916827176</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1899605649867625</v>
+        <v>0.04727718438101908</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1709645084880862</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.1282233813660647</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.08242931659247014</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.04636649058326446</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.02318324529163223</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.0104324603812345</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.004267824701414115</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.001600434263030293</v>
+        <v>0.01418315531430573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tilføjet plots for både solutiob og path simulering
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,31 @@
           <t>demand_5</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>demand_6</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>demand_7</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>demand_8</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>demand_9</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>demand_10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -467,22 +492,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.085685596340511</v>
+        <v>0.08209005758049948</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2142139908512775</v>
+        <v>0.2052251439512487</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2677674885640969</v>
+        <v>0.2565314299390609</v>
       </c>
       <c r="E2" t="n">
-        <v>0.223139573803414</v>
+        <v>0.213776191615884</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1394622336271338</v>
+        <v>0.1336101197599275</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06973111681356689</v>
+        <v>0.06680505987996375</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.02783544161665157</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.009941229148804132</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.003106634109001291</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0008629539191670253</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0002157384797917563</v>
       </c>
     </row>
     <row r="3">
@@ -492,22 +532,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.03521094473532189</v>
+        <v>0.03022819787909564</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1232383065736266</v>
+        <v>0.1057986925768347</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2156670365038466</v>
+        <v>0.1851477120094608</v>
       </c>
       <c r="E3" t="n">
-        <v>0.251611542587821</v>
+        <v>0.2160056640110376</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2201600997643434</v>
+        <v>0.1890049560096579</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1541120698350404</v>
+        <v>0.1323034692067605</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.07717702370394364</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.03858851185197182</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.01688247393523767</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.006565406530370205</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.002297892285629572</v>
       </c>
     </row>
     <row r="4">
@@ -517,22 +572,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02332814930015552</v>
+        <v>0.0183677991424473</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0933125972006221</v>
+        <v>0.07347119656978922</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1866251944012442</v>
+        <v>0.1469423931395784</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2488335925349922</v>
+        <v>0.1959231908527712</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2488335925349922</v>
+        <v>0.1959231908527712</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1990668740279938</v>
+        <v>0.156738552682217</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1044923684548113</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.05970992483132077</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.02985496241566038</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.01326887218473795</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.005307548873895179</v>
       </c>
     </row>
     <row r="5">
@@ -542,22 +612,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.03521094473532189</v>
+        <v>0.03022819787909564</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1232383065736266</v>
+        <v>0.1057986925768347</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2156670365038466</v>
+        <v>0.1851477120094608</v>
       </c>
       <c r="E5" t="n">
-        <v>0.251611542587821</v>
+        <v>0.2160056640110376</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2201600997643434</v>
+        <v>0.1890049560096579</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1541120698350404</v>
+        <v>0.1323034692067605</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.07717702370394364</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.03858851185197182</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.01688247393523767</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.006565406530370205</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.002297892285629572</v>
       </c>
     </row>
     <row r="6">
@@ -567,22 +652,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.05434782608695652</v>
+        <v>0.04980162722370379</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1630434782608696</v>
+        <v>0.1494048816711114</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2445652173913044</v>
+        <v>0.2241073225066671</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2445652173913044</v>
+        <v>0.2241073225066671</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1834239130434783</v>
+        <v>0.1680804918800003</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1100543478260869</v>
+        <v>0.1008482951280002</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.05042414756400009</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.02161034895600004</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.008103880858500015</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.002701293619500005</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.0008103880858500015</v>
       </c>
     </row>
     <row r="7">
@@ -592,22 +692,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1376146788990826</v>
+        <v>0.1353364076418526</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2752293577981652</v>
+        <v>0.2706728152837052</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2752293577981652</v>
+        <v>0.2706728152837052</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1834862385321101</v>
+        <v>0.1804485435224701</v>
       </c>
       <c r="F7" t="n">
-        <v>0.09174311926605505</v>
+        <v>0.09022427176123507</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03669724770642202</v>
+        <v>0.03608970870449403</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.01202990290149801</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.003437115114713717</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.0008592787786784291</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.0001909508397063176</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3.819016794126351e-05</v>
       </c>
     </row>
     <row r="8">
@@ -617,22 +732,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.224128874102609</v>
+        <v>0.2231302832612856</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3361933111539135</v>
+        <v>0.3346954248919284</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2521449833654351</v>
+        <v>0.2510215686689463</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1260724916827176</v>
+        <v>0.1255107843344732</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04727718438101908</v>
+        <v>0.04706654412542743</v>
       </c>
       <c r="G8" t="n">
-        <v>0.01418315531430573</v>
+        <v>0.01411996323762823</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.003529990809407058</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.000756426602015798</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.0001418299878779621</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.363833131299369e-05</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.545749696949053e-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Justeret cost variabler og tilføjet fixed demand + stokastisk støj
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DemandProbabilities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeekdayBaseDemand" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoiseDistribution" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,26 +467,6 @@
           <t>demand_6</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>demand_7</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>demand_8</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>demand_9</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>demand_10</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -492,37 +475,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.08209005758049948</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2052251439512487</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2565314299390609</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.213776191615884</v>
+        <v>0.260597637248089</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1336101197599275</v>
+        <v>0.3648366921473246</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06680505987996375</v>
+        <v>0.2553856845031272</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02783544161665157</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.009941229148804132</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.003106634109001291</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.0008629539191670253</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.0002157384797917563</v>
+        <v>0.1191799861014594</v>
       </c>
     </row>
     <row r="3">
@@ -532,37 +503,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.03022819787909564</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1057986925768347</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1851477120094608</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2160056640110376</v>
+        <v>0.2848056201642379</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1890049560096579</v>
+        <v>0.3702473062135093</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1323034692067605</v>
+        <v>0.240660749038781</v>
       </c>
       <c r="H3" t="n">
-        <v>0.07717702370394364</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.03858851185197182</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.01688247393523767</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.006565406530370205</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.002297892285629572</v>
+        <v>0.1042863245834718</v>
       </c>
     </row>
     <row r="4">
@@ -572,37 +531,25 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0183677991424473</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>0.07347119656978922</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1469423931395784</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1959231908527712</v>
+        <v>0.3117206982543641</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1959231908527712</v>
+        <v>0.374064837905237</v>
       </c>
       <c r="G4" t="n">
-        <v>0.156738552682217</v>
+        <v>0.2244389027431422</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1044923684548113</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.05970992483132077</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.02985496241566038</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.01326887218473795</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.005307548873895179</v>
+        <v>0.08977556109725686</v>
       </c>
     </row>
     <row r="5">
@@ -612,37 +559,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.03022819787909564</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1057986925768347</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1851477120094608</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2160056640110376</v>
+        <v>0.260597637248089</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1890049560096579</v>
+        <v>0.3648366921473246</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1323034692067605</v>
+        <v>0.2553856845031272</v>
       </c>
       <c r="H5" t="n">
-        <v>0.07717702370394364</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.03858851185197182</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.01688247393523767</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.006565406530370205</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.002297892285629572</v>
+        <v>0.1191799861014594</v>
       </c>
     </row>
     <row r="6">
@@ -652,37 +587,25 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.04980162722370379</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1494048816711114</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2241073225066671</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2241073225066671</v>
+        <v>0.3117206982543641</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1680804918800003</v>
+        <v>0.374064837905237</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1008482951280002</v>
+        <v>0.2244389027431422</v>
       </c>
       <c r="H6" t="n">
-        <v>0.05042414756400009</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.02161034895600004</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.008103880858500015</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.002701293619500005</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.0008103880858500015</v>
+        <v>0.08977556109725686</v>
       </c>
     </row>
     <row r="7">
@@ -692,37 +615,25 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1353364076418526</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2706728152837052</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2706728152837052</v>
+        <v>0.4534461910519951</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1804485435224701</v>
+        <v>0.3627569528415961</v>
       </c>
       <c r="F7" t="n">
-        <v>0.09022427176123507</v>
+        <v>0.1451027811366385</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03608970870449403</v>
+        <v>0.03869407496977027</v>
       </c>
       <c r="H7" t="n">
-        <v>0.01202990290149801</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.003437115114713717</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.0008592787786784291</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.0001909508397063176</v>
-      </c>
-      <c r="L7" t="n">
-        <v>3.819016794126351e-05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -732,37 +643,449 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.2231302832612856</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.3346954248919284</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2510215686689463</v>
+        <v>0.41211621677313</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1255107843344732</v>
+        <v>0.370904595095817</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04706654412542743</v>
+        <v>0.1669070677931177</v>
       </c>
       <c r="G8" t="n">
-        <v>0.01411996323762823</v>
+        <v>0.0500721203379353</v>
       </c>
       <c r="H8" t="n">
-        <v>0.003529990809407058</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.000756426602015798</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.0001418299878779621</v>
-      </c>
-      <c r="K8" t="n">
-        <v>2.363833131299369e-05</v>
-      </c>
-      <c r="L8" t="n">
-        <v>3.545749696949053e-06</v>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>weekday</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>weekday_weight</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>weekday_mean_before_rounding</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>base_demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.921102739726028</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.921102739726028</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.788325342465754</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.788325342465754</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.65554794520548</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.257215753424658</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.257215753424658</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>weekday</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>noise_lambda</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_0</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.260597637248089</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.3648366921473246</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2553856845031272</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1191799861014594</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2848056201642379</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.3702473062135093</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.240660749038781</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.1042863245834718</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.3117206982543641</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.374064837905237</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2244389027431422</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.08977556109725686</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.260597637248089</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.3648366921473246</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.2553856845031272</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1191799861014594</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.3117206982543641</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.374064837905237</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.2244389027431422</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.08977556109725686</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.4534461910519951</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.3627569528415961</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.1451027811366385</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.03869407496977027</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.41211621677313</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.370904595095817</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.1669070677931177</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0500721203379353</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>annual_total_products</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7754.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>units_per_model_unit</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>average_daily_demand_in_model_units</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.65554794520548</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>max_noise</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Parametre til policy analyse er fundet: inventory cap 15, max order 9, shelf life 5, c_outdate og c_production 2500, c_hold 5 og c_shortage 20000
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,21 @@
           <t>demand_6</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>demand_7</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>demand_8</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>demand_9</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -484,16 +499,25 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.260597637248089</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3648366921473246</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2553856845031272</v>
+        <v>0.3117206982543641</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1191799861014594</v>
+        <v>0.3740648379052369</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.2244389027431422</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.08977556109725685</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -512,16 +536,25 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.2848056201642379</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.3702473062135093</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.240660749038781</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.1042863245834718</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -540,16 +573,25 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.3117206982543641</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.374064837905237</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2244389027431422</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0.08977556109725686</v>
+        <v>0.260597637248089</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.3648366921473246</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.2553856845031272</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1191799861014593</v>
       </c>
     </row>
     <row r="5">
@@ -568,16 +610,25 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.260597637248089</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3648366921473246</v>
+        <v>0.2848056201642379</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2553856845031272</v>
+        <v>0.3702473062135093</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1191799861014594</v>
+        <v>0.240660749038781</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.1042863245834718</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -596,16 +647,25 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.3117206982543641</v>
       </c>
-      <c r="F6" t="n">
-        <v>0.374064837905237</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
+        <v>0.3740648379052369</v>
+      </c>
+      <c r="I6" t="n">
         <v>0.2244389027431422</v>
       </c>
-      <c r="H6" t="n">
-        <v>0.08977556109725686</v>
+      <c r="J6" t="n">
+        <v>0.08977556109725685</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -618,21 +678,30 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.6075949367088608</v>
       </c>
       <c r="D7" t="n">
-        <v>0.4534461910519951</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3627569528415961</v>
+        <v>0.0759493670886076</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1451027811366385</v>
+        <v>0.01265822784810127</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03869407496977027</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -646,21 +715,30 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.5506607929515418</v>
       </c>
       <c r="D8" t="n">
-        <v>0.41211621677313</v>
+        <v>0.3303964757709251</v>
       </c>
       <c r="E8" t="n">
-        <v>0.370904595095817</v>
+        <v>0.09911894273127753</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1669070677931177</v>
+        <v>0.0198237885462555</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0500721203379353</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -707,13 +785,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.1</v>
+        <v>24</v>
       </c>
       <c r="C2" t="n">
-        <v>2.921102739726028</v>
+        <v>4.720974124809741</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -723,13 +801,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.1</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>2.921102739726028</v>
+        <v>3.737437848807712</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -739,13 +817,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.05</v>
+        <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>2.788325342465754</v>
+        <v>5.901217656012177</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -755,13 +833,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.05</v>
+        <v>18</v>
       </c>
       <c r="C5" t="n">
-        <v>2.788325342465754</v>
+        <v>3.540730593607306</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -771,13 +849,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C6" t="n">
-        <v>2.65554794520548</v>
+        <v>4.524266869609335</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -787,13 +865,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.85</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>2.257215753424658</v>
+        <v>0.9835362760020294</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -803,13 +881,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.85</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>2.257215753424658</v>
+        <v>1.376950786402841</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -865,19 +943,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="C2" t="n">
-        <v>0.260597637248089</v>
+        <v>0.3117206982543641</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3648366921473246</v>
+        <v>0.3740648379052369</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2553856845031272</v>
+        <v>0.2244389027431422</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1191799861014594</v>
+        <v>0.08977556109725685</v>
       </c>
     </row>
     <row r="3">
@@ -909,19 +987,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3117206982543641</v>
+        <v>0.260597637248089</v>
       </c>
       <c r="D4" t="n">
-        <v>0.374064837905237</v>
+        <v>0.3648366921473246</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2244389027431422</v>
+        <v>0.2553856845031272</v>
       </c>
       <c r="F4" t="n">
-        <v>0.08977556109725686</v>
+        <v>0.1191799861014593</v>
       </c>
     </row>
     <row r="5">
@@ -931,19 +1009,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="C5" t="n">
-        <v>0.260597637248089</v>
+        <v>0.2848056201642379</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3648366921473246</v>
+        <v>0.3702473062135093</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2553856845031272</v>
+        <v>0.240660749038781</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1191799861014594</v>
+        <v>0.1042863245834718</v>
       </c>
     </row>
     <row r="6">
@@ -959,13 +1037,13 @@
         <v>0.3117206982543641</v>
       </c>
       <c r="D6" t="n">
-        <v>0.374064837905237</v>
+        <v>0.3740648379052369</v>
       </c>
       <c r="E6" t="n">
         <v>0.2244389027431422</v>
       </c>
       <c r="F6" t="n">
-        <v>0.08977556109725686</v>
+        <v>0.08977556109725685</v>
       </c>
     </row>
     <row r="7">
@@ -975,19 +1053,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4534461910519951</v>
+        <v>0.6075949367088608</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3627569528415961</v>
+        <v>0.3037974683544304</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1451027811366385</v>
+        <v>0.0759493670886076</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03869407496977027</v>
+        <v>0.01265822784810127</v>
       </c>
     </row>
     <row r="8">
@@ -997,19 +1075,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="C8" t="n">
-        <v>0.41211621677313</v>
+        <v>0.5506607929515418</v>
       </c>
       <c r="D8" t="n">
-        <v>0.370904595095817</v>
+        <v>0.3303964757709251</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1669070677931177</v>
+        <v>0.09911894273127753</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0500721203379353</v>
+        <v>0.0198237885462555</v>
       </c>
     </row>
   </sheetData>
@@ -1055,7 +1133,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -1065,7 +1143,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.65554794520548</v>
+        <v>3.540730593607306</v>
       </c>
     </row>
     <row r="5">
@@ -1085,7 +1163,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fjernet infeasible states fra simulerings-scriptet
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:AD8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,101 @@
           <t>demand_9</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>demand_10</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>demand_11</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>demand_12</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>demand_13</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>demand_14</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>demand_15</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>demand_16</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>demand_17</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>demand_18</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>demand_19</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>demand_20</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>demand_21</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>demand_22</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>demand_23</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>demand_24</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>demand_25</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>demand_26</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>demand_27</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>demand_28</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -505,18 +600,75 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3117206982543641</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3740648379052369</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2244389027431422</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.08977556109725685</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0450664812557408</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.1397060918927965</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.2165444424338346</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.2237625905149624</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.1734160076490958</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.1075179247424394</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0555509277835937</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.02460112516130579</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.009532936000005992</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.003283566844446509</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.001017905721778418</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -539,21 +691,78 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2848056201642379</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3702473062135093</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.240660749038781</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1042863245834718</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.06721358191961016</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.1814766711829474</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.2449935060969791</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.2204941554872812</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.1488335549539148</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.08037011967511401</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.0361665538538013</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.01394995648646622</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.004708110314182348</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.001412433094254705</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.0003813569354487703</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -582,16 +791,73 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0.260597637248089</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0.3648366921473246</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.2553856845031272</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1191799861014593</v>
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.01662938425914923</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.06818047546251182</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.1397699746981492</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1910189654208039</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.195794439556324</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0.1605514404361857</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0.1097101509647269</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0.06425880270791146</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.03293263638780461</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>0.01500264546555543</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.006151084640877727</v>
       </c>
     </row>
     <row r="5">
@@ -613,21 +879,78 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2848056201642379</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3702473062135093</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.240660749038781</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1042863245834718</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.05503533924501622</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.159602483810547</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.2314236015252932</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.2237094814744501</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.1621893740689763</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.09406983696000626</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.04546708786400301</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.01883636497222982</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.006828182302433311</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.002200192075228511</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.0006380557018162682</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -653,18 +976,75 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3117206982543641</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3740648379052369</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2244389027431422</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0.08977556109725685</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.07428001934180856</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.1931280502887023</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.251066465375313</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.2175909366586045</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.141434108828093</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.07354573659060834</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.03186981918926361</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.01183736141315506</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.003847142459275395</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.001111396710457336</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.0002889631447189074</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -678,30 +1058,87 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6075949367088608</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3037974683544304</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0759493670886076</v>
+        <v>0.2231302832612856</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01265822784810127</v>
+        <v>0.3346954248919284</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>0.2510215686689463</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>0.1255107843344732</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>0.04706654412542743</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>0.01411996323762823</v>
       </c>
       <c r="K7" t="n">
+        <v>0.003529990809407058</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.000756426602015798</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.0001418299878779621</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2.363833131299369e-05</v>
+      </c>
+      <c r="O7" t="n">
+        <v>3.545749696949053e-06</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -715,30 +1152,87 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5506607929515418</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3303964757709251</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0.09911894273127753</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0198237885462555</v>
+        <v>0.2018967249205256</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>0.323034759872841</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>0.2584278078982729</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.1378281642124122</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>0.05513126568496488</v>
       </c>
       <c r="K8" t="n">
+        <v>0.01764200501918876</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.00470453467178367</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.00107532221069341</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.0002150644421386821</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3.823367860243238e-05</v>
+      </c>
+      <c r="P8" t="n">
+        <v>6.11738857638918e-06</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -788,10 +1282,10 @@
         <v>24</v>
       </c>
       <c r="C2" t="n">
-        <v>4.720974124809741</v>
+        <v>14.16292237442922</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -804,10 +1298,10 @@
         <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>3.737437848807712</v>
+        <v>11.21231354642314</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -820,10 +1314,10 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>5.901217656012177</v>
+        <v>17.70365296803653</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -836,10 +1330,10 @@
         <v>18</v>
       </c>
       <c r="C5" t="n">
-        <v>3.540730593607306</v>
+        <v>10.62219178082192</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -852,10 +1346,10 @@
         <v>23</v>
       </c>
       <c r="C6" t="n">
-        <v>4.524266869609335</v>
+        <v>13.57280060882801</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -868,10 +1362,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9835362760020294</v>
+        <v>2.950608828006088</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -884,10 +1378,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>1.376950786402841</v>
+        <v>4.130852359208524</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -901,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,6 +1429,41 @@
           <t>P_noise_3</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_4</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_5</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_6</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_7</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_8</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_9</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>P_noise_10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -943,19 +1472,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.2</v>
+        <v>3.1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3117206982543641</v>
+        <v>0.0450664812557408</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3740648379052369</v>
+        <v>0.1397060918927965</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2244389027431422</v>
+        <v>0.2165444424338346</v>
       </c>
       <c r="F2" t="n">
-        <v>0.08977556109725685</v>
+        <v>0.2237625905149624</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.1734160076490958</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.1075179247424394</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0555509277835937</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.02460112516130579</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.009532936000005992</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.003283566844446509</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.001017905721778418</v>
       </c>
     </row>
     <row r="3">
@@ -965,19 +1515,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.3</v>
+        <v>2.7</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2848056201642379</v>
+        <v>0.06721358191961016</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3702473062135093</v>
+        <v>0.1814766711829474</v>
       </c>
       <c r="E3" t="n">
-        <v>0.240660749038781</v>
+        <v>0.2449935060969791</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1042863245834718</v>
+        <v>0.2204941554872812</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.1488335549539148</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.08037011967511401</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.0361665538538013</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.01394995648646622</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.004708110314182348</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.001412433094254705</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.0003813569354487703</v>
       </c>
     </row>
     <row r="4">
@@ -987,19 +1558,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.4</v>
+        <v>4.1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.260597637248089</v>
+        <v>0.01662938425914923</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3648366921473246</v>
+        <v>0.06818047546251182</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2553856845031272</v>
+        <v>0.1397699746981492</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1191799861014593</v>
+        <v>0.1910189654208039</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.195794439556324</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.1605514404361857</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1097101509647269</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.06425880270791146</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.03293263638780461</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.01500264546555543</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.006151084640877727</v>
       </c>
     </row>
     <row r="5">
@@ -1009,19 +1601,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.3</v>
+        <v>2.9</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2848056201642379</v>
+        <v>0.05503533924501622</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3702473062135093</v>
+        <v>0.159602483810547</v>
       </c>
       <c r="E5" t="n">
-        <v>0.240660749038781</v>
+        <v>0.2314236015252932</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1042863245834718</v>
+        <v>0.2237094814744501</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1621893740689763</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.09406983696000626</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.04546708786400301</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.01883636497222982</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.006828182302433311</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.002200192075228511</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.0006380557018162682</v>
       </c>
     </row>
     <row r="6">
@@ -1031,19 +1644,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.2</v>
+        <v>2.6</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3117206982543641</v>
+        <v>0.07428001934180856</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3740648379052369</v>
+        <v>0.1931280502887023</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2244389027431422</v>
+        <v>0.251066465375313</v>
       </c>
       <c r="F6" t="n">
-        <v>0.08977556109725685</v>
+        <v>0.2175909366586045</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.141434108828093</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.07354573659060834</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.03186981918926361</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.01183736141315506</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.003847142459275395</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.001111396710457336</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.0002889631447189074</v>
       </c>
     </row>
     <row r="7">
@@ -1053,19 +1687,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C7" t="n">
-        <v>0.6075949367088608</v>
+        <v>0.2231302832612856</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3037974683544304</v>
+        <v>0.3346954248919284</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0759493670886076</v>
+        <v>0.2510215686689463</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01265822784810127</v>
+        <v>0.1255107843344732</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.04706654412542743</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.01411996323762823</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.003529990809407058</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.000756426602015798</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.0001418299878779621</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.363833131299369e-05</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3.545749696949053e-06</v>
       </c>
     </row>
     <row r="8">
@@ -1075,19 +1730,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.6</v>
+        <v>1.6</v>
       </c>
       <c r="C8" t="n">
-        <v>0.5506607929515418</v>
+        <v>0.2018967249205256</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3303964757709251</v>
+        <v>0.323034759872841</v>
       </c>
       <c r="E8" t="n">
-        <v>0.09911894273127753</v>
+        <v>0.2584278078982729</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0198237885462555</v>
+        <v>0.1378281642124122</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.05513126568496488</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.01764200501918876</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00470453467178367</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.00107532221069341</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.0002150644421386821</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3.823367860243238e-05</v>
+      </c>
+      <c r="M8" t="n">
+        <v>6.11738857638918e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1133,7 +1809,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1143,7 +1819,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.540730593607306</v>
+        <v>10.62219178082192</v>
       </c>
     </row>
     <row r="5">
@@ -1153,7 +1829,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -1163,7 +1839,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nyt script til demand distribution generation
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DemandProbabilities" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeekdayBaseDemand" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoiseDistribution" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WeekdayCenteredDemand" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CenteredPoissonOffset" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD8"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -557,26 +557,6 @@
           <t>demand_24</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>demand_25</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>demand_26</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>demand_27</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>demand_28</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -627,49 +607,37 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0450664812557408</v>
+        <v>0.01041935654618319</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1397060918927965</v>
+        <v>0.04763277420099123</v>
       </c>
       <c r="R2" t="n">
-        <v>0.2165444424338346</v>
+        <v>0.1088781811058069</v>
       </c>
       <c r="S2" t="n">
-        <v>0.2237625905149624</v>
+        <v>0.165914590248132</v>
       </c>
       <c r="T2" t="n">
-        <v>0.1734160076490958</v>
+        <v>0.1896223672476748</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1075179247424394</v>
+        <v>0.1733742263743649</v>
       </c>
       <c r="V2" t="n">
-        <v>0.0555509277835937</v>
+        <v>0.1320986144163069</v>
       </c>
       <c r="W2" t="n">
-        <v>0.02460112516130579</v>
+        <v>0.08627107283950429</v>
       </c>
       <c r="X2" t="n">
-        <v>0.009532936000005992</v>
+        <v>0.04929923592722601</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.003283566844446509</v>
+        <v>0.02504163351903341</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.001017905721778418</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0</v>
+        <v>0.01144794757477647</v>
       </c>
     </row>
     <row r="3">
@@ -712,57 +680,45 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.06721358191961016</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1814766711829474</v>
+        <v>0.006302111920819578</v>
       </c>
       <c r="O3" t="n">
-        <v>0.2449935060969791</v>
+        <v>0.03202882452620821</v>
       </c>
       <c r="P3" t="n">
-        <v>0.2204941554872812</v>
+        <v>0.08138903382068369</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.1488335549539148</v>
+        <v>0.1378794450364344</v>
       </c>
       <c r="R3" t="n">
-        <v>0.08037011967511401</v>
+        <v>0.1751839941248069</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0361665538538013</v>
+        <v>0.1780653050317151</v>
       </c>
       <c r="T3" t="n">
-        <v>0.01394995648646622</v>
+        <v>0.1508283382016075</v>
       </c>
       <c r="U3" t="n">
-        <v>0.004708110314182348</v>
+        <v>0.1095064738055672</v>
       </c>
       <c r="V3" t="n">
-        <v>0.001412433094254705</v>
+        <v>0.06956722758317427</v>
       </c>
       <c r="W3" t="n">
-        <v>0.0003813569354487703</v>
+        <v>0.03928412416929229</v>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>0.01996512177969077</v>
       </c>
       <c r="Y3" t="n">
         <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -806,58 +762,46 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>0.007757224322108526</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>0.03778307833437945</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>0.0920149366025954</v>
       </c>
       <c r="P4" t="n">
-        <v>0</v>
+        <v>0.1493922487918904</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>0.1819110420258816</v>
       </c>
       <c r="R4" t="n">
-        <v>0</v>
+        <v>0.177206662211987</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>0.1438532848372736</v>
       </c>
       <c r="T4" t="n">
-        <v>0.01662938425914923</v>
+        <v>0.10009508010992</v>
       </c>
       <c r="U4" t="n">
-        <v>0.06818047546251182</v>
+        <v>0.06094158322037407</v>
       </c>
       <c r="V4" t="n">
-        <v>0.1397699746981492</v>
+        <v>0.03298087788199748</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1910189654208039</v>
+        <v>0.01606398166159259</v>
       </c>
       <c r="X4" t="n">
-        <v>0.195794439556324</v>
+        <v>0</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.1605514404361857</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.1097101509647269</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0.06425880270791146</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0.03293263638780461</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>0.01500264546555543</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.006151084640877727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -900,57 +844,45 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.05503533924501622</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.159602483810547</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2314236015252932</v>
+        <v>0.005782510694012257</v>
       </c>
       <c r="P5" t="n">
-        <v>0.2237094814744501</v>
+        <v>0.02989624855565904</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.1621893740689763</v>
+        <v>0.07728353002677996</v>
       </c>
       <c r="R5" t="n">
-        <v>0.09406983696000626</v>
+        <v>0.1331882605556235</v>
       </c>
       <c r="S5" t="n">
-        <v>0.04546708786400301</v>
+        <v>0.1721496748112352</v>
       </c>
       <c r="T5" t="n">
-        <v>0.01883636497222982</v>
+        <v>0.1780067427203154</v>
       </c>
       <c r="U5" t="n">
-        <v>0.006828182302433311</v>
+        <v>0.1533859052625823</v>
       </c>
       <c r="V5" t="n">
-        <v>0.002200192075228511</v>
+        <v>0.1132889795088329</v>
       </c>
       <c r="W5" t="n">
-        <v>0.0006380557018162682</v>
+        <v>0.0732146395665155</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>0.04205868308418859</v>
       </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>0.02174482521425543</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -997,54 +929,42 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>0.003886828339677544</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>0.02168111527932997</v>
       </c>
       <c r="P6" t="n">
-        <v>0.07428001934180856</v>
+        <v>0.06046970932019514</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.1931280502887023</v>
+        <v>0.1124353520920257</v>
       </c>
       <c r="R6" t="n">
-        <v>0.251066465375313</v>
+        <v>0.1567938957642197</v>
       </c>
       <c r="S6" t="n">
-        <v>0.2175909366586045</v>
+        <v>0.1749223908067583</v>
       </c>
       <c r="T6" t="n">
-        <v>0.141434108828093</v>
+        <v>0.1626224172419531</v>
       </c>
       <c r="U6" t="n">
-        <v>0.07354573659060834</v>
+        <v>0.129589146695176</v>
       </c>
       <c r="V6" t="n">
-        <v>0.03186981918926361</v>
+        <v>0.09035764455323243</v>
       </c>
       <c r="W6" t="n">
-        <v>0.01183736141315506</v>
+        <v>0.05600265925844766</v>
       </c>
       <c r="X6" t="n">
-        <v>0.003847142459275395</v>
+        <v>0.03123884064898455</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.001111396710457336</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.0002889631447189074</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1064,49 +984,49 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2231302832612856</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3346954248919284</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2510215686689463</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1255107843344732</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.04706654412542743</v>
+        <v>0.008832005957155406</v>
       </c>
       <c r="J7" t="n">
-        <v>0.01411996323762823</v>
+        <v>0.04185457976831192</v>
       </c>
       <c r="K7" t="n">
-        <v>0.003529990809407058</v>
+        <v>0.09917372429774736</v>
       </c>
       <c r="L7" t="n">
-        <v>0.000756426602015798</v>
+        <v>0.1566603168323928</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0001418299878779621</v>
+        <v>0.1856019957187125</v>
       </c>
       <c r="N7" t="n">
-        <v>2.363833131299369e-05</v>
+        <v>0.1759123255272064</v>
       </c>
       <c r="O7" t="n">
-        <v>3.545749696949053e-06</v>
+        <v>0.1389404343083703</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>0.09406200777060039</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>0.05571958718240842</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>0.02933925036958104</v>
       </c>
       <c r="S7" t="n">
-        <v>0</v>
+        <v>0.0139037722675134</v>
       </c>
       <c r="T7" t="n">
         <v>0</v>
@@ -1127,18 +1047,6 @@
         <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1161,43 +1069,43 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2018967249205256</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0.323034759872841</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2584278078982729</v>
+        <v>0.008832005957155406</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1378281642124122</v>
+        <v>0.04185457976831192</v>
       </c>
       <c r="J8" t="n">
-        <v>0.05513126568496488</v>
+        <v>0.09917372429774736</v>
       </c>
       <c r="K8" t="n">
-        <v>0.01764200501918876</v>
+        <v>0.1566603168323928</v>
       </c>
       <c r="L8" t="n">
-        <v>0.00470453467178367</v>
+        <v>0.1856019957187125</v>
       </c>
       <c r="M8" t="n">
-        <v>0.00107532221069341</v>
+        <v>0.1759123255272064</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0002150644421386821</v>
+        <v>0.1389404343083703</v>
       </c>
       <c r="O8" t="n">
-        <v>3.823367860243238e-05</v>
+        <v>0.09406200777060039</v>
       </c>
       <c r="P8" t="n">
-        <v>6.11738857638918e-06</v>
+        <v>0.05571958718240842</v>
       </c>
       <c r="Q8" t="n">
-        <v>0</v>
+        <v>0.02933925036958104</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>0.0139037722675134</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
@@ -1221,18 +1129,6 @@
         <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1247,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1258,17 +1154,77 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>weekday_weight</t>
+          <t>annual_demand_real_units</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>weekday_mean_before_rounding</t>
+          <t>number_of_weekdays_in_year</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>base_demand</t>
+          <t>mean_real_units_per_day</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mean_model_units_per_day</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>base_demand_nearest_integer</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>max_noise_full_width_model_units</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>lower_demand_model_units</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>upper_demand_model_units</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>target_offset_mean_model_units</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>fitted_truncated_poisson_lambda</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>expected_offset_model_units</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>expected_total_model_units</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>expected_total_real_units</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>signed_deviation_min_from_nearest_base</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>signed_deviation_max_from_nearest_base</t>
         </is>
       </c>
     </row>
@@ -1279,13 +1235,49 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>963</v>
+      </c>
+      <c r="C2" t="n">
+        <v>52</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18.51923076923077</v>
+      </c>
+      <c r="E2" t="n">
+        <v>18.51923076923077</v>
+      </c>
+      <c r="F2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G2" t="n">
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
+        <v>14</v>
+      </c>
+      <c r="I2" t="n">
         <v>24</v>
       </c>
-      <c r="C2" t="n">
-        <v>14.16292237442922</v>
-      </c>
-      <c r="D2" t="n">
-        <v>14</v>
+      <c r="J2" t="n">
+        <v>4.51923076923077</v>
+      </c>
+      <c r="K2" t="n">
+        <v>4.57156581501571</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4.519230769230769</v>
+      </c>
+      <c r="M2" t="n">
+        <v>18.51923076923077</v>
+      </c>
+      <c r="N2" t="n">
+        <v>18.51923076923077</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -1295,13 +1287,49 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>883</v>
       </c>
       <c r="C3" t="n">
-        <v>11.21231354642314</v>
+        <v>52</v>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>16.98076923076923</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16.98076923076923</v>
+      </c>
+      <c r="F3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I3" t="n">
+        <v>22</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4.98076923076923</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.08223670550791</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.98076923076923</v>
+      </c>
+      <c r="M3" t="n">
+        <v>16.98076923076923</v>
+      </c>
+      <c r="N3" t="n">
+        <v>16.98076923076923</v>
+      </c>
+      <c r="O3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1311,13 +1339,49 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30</v>
+        <v>837</v>
       </c>
       <c r="C4" t="n">
-        <v>17.70365296803653</v>
+        <v>53</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>15.79245283018868</v>
+      </c>
+      <c r="E4" t="n">
+        <v>15.79245283018868</v>
+      </c>
+      <c r="F4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4.79245283018868</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4.870695594904424</v>
+      </c>
+      <c r="L4" t="n">
+        <v>4.79245283018868</v>
+      </c>
+      <c r="M4" t="n">
+        <v>15.79245283018868</v>
+      </c>
+      <c r="N4" t="n">
+        <v>15.79245283018868</v>
+      </c>
+      <c r="O4" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1327,13 +1391,49 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>939</v>
+      </c>
+      <c r="C5" t="n">
+        <v>52</v>
+      </c>
+      <c r="D5" t="n">
+        <v>18.05769230769231</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18.05769230769231</v>
+      </c>
+      <c r="F5" t="n">
         <v>18</v>
       </c>
-      <c r="C5" t="n">
-        <v>10.62219178082192</v>
-      </c>
-      <c r="D5" t="n">
-        <v>11</v>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>13</v>
+      </c>
+      <c r="I5" t="n">
+        <v>23</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5.057692307692307</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5.170115567034983</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5.057692307692307</v>
+      </c>
+      <c r="M5" t="n">
+        <v>18.05769230769231</v>
+      </c>
+      <c r="N5" t="n">
+        <v>18.05769230769231</v>
+      </c>
+      <c r="O5" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -1343,13 +1443,49 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>23</v>
+        <v>905</v>
       </c>
       <c r="C6" t="n">
-        <v>13.57280060882801</v>
+        <v>52</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>17.40384615384615</v>
+      </c>
+      <c r="E6" t="n">
+        <v>17.40384615384615</v>
+      </c>
+      <c r="F6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" t="n">
+        <v>22</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5.403846153846153</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5.578099515742613</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5.403846153846152</v>
+      </c>
+      <c r="M6" t="n">
+        <v>17.40384615384615</v>
+      </c>
+      <c r="N6" t="n">
+        <v>17.40384615384615</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1359,13 +1495,49 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>607</v>
+      </c>
+      <c r="C7" t="n">
+        <v>52</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11.67307692307692</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11.67307692307692</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" t="n">
+        <v>17</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4.673076923076923</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4.738966433146786</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4.673076923076922</v>
+      </c>
+      <c r="M7" t="n">
+        <v>11.67307692307692</v>
+      </c>
+      <c r="N7" t="n">
+        <v>11.67307692307692</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P7" t="n">
         <v>5</v>
-      </c>
-      <c r="C7" t="n">
-        <v>2.950608828006088</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1375,13 +1547,49 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>555</v>
       </c>
       <c r="C8" t="n">
-        <v>4.130852359208524</v>
+        <v>52</v>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>10.67307692307692</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10.67307692307692</v>
+      </c>
+      <c r="F8" t="n">
+        <v>11</v>
+      </c>
+      <c r="G8" t="n">
+        <v>10</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>16</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4.673076923076923</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4.738966433146786</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4.673076923076922</v>
+      </c>
+      <c r="M8" t="n">
+        <v>10.67307692307692</v>
+      </c>
+      <c r="N8" t="n">
+        <v>10.67307692307692</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-5</v>
+      </c>
+      <c r="P8" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1395,7 +1603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:BT8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1406,62 +1614,357 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>noise_lambda</t>
+          <t>lower_demand_model_units</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_0</t>
+          <t>upper_demand_model_units</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_1</t>
+          <t>target_offset_mean_model_units</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_2</t>
+          <t>fitted_truncated_poisson_lambda</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_3</t>
+          <t>expected_total_model_units</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_4</t>
+          <t>P_offset_0_demand_14</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_5</t>
+          <t>P_offset_1_demand_15</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_6</t>
+          <t>P_offset_2_demand_16</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_7</t>
+          <t>P_offset_3_demand_17</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_8</t>
+          <t>P_offset_4_demand_18</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_9</t>
+          <t>P_offset_5_demand_19</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>P_noise_10</t>
+          <t>P_offset_6_demand_20</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_21</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_22</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_23</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_24</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_12</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_13</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_14</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_15</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_16</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_17</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_18</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_19</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_20</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_21</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_22</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_11</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_12</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_13</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_14</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_15</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_16</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_17</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_18</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_19</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_20</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_21</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_13</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_14</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_15</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_16</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_17</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_18</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_19</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_20</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_21</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_22</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_23</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_7</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_8</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_9</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_10</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_11</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_12</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_13</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_14</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_15</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_16</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_17</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_0_demand_6</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_1_demand_7</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_2_demand_8</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_3_demand_9</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_4_demand_10</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_5_demand_11</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_6_demand_12</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_7_demand_13</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_8_demand_14</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_9_demand_15</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>P_offset_10_demand_16</t>
         </is>
       </c>
     </row>
@@ -1472,41 +1975,108 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.1</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0450664812557408</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1397060918927965</v>
+        <v>4.51923076923077</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2165444424338346</v>
+        <v>4.57156581501571</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2237625905149624</v>
+        <v>18.51923076923077</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1734160076490958</v>
+        <v>0.01041935654618319</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1075179247424394</v>
+        <v>0.04763277420099123</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0555509277835937</v>
+        <v>0.1088781811058069</v>
       </c>
       <c r="J2" t="n">
-        <v>0.02460112516130579</v>
+        <v>0.165914590248132</v>
       </c>
       <c r="K2" t="n">
-        <v>0.009532936000005992</v>
+        <v>0.1896223672476748</v>
       </c>
       <c r="L2" t="n">
-        <v>0.003283566844446509</v>
+        <v>0.1733742263743649</v>
       </c>
       <c r="M2" t="n">
-        <v>0.001017905721778418</v>
-      </c>
+        <v>0.1320986144163069</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.08627107283950429</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.04929923592722601</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.02504163351903341</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.01144794757477647</v>
+      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1515,41 +2085,108 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.7</v>
+        <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06721358191961016</v>
+        <v>22</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1814766711829474</v>
+        <v>4.98076923076923</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2449935060969791</v>
+        <v>5.08223670550791</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2204941554872812</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.1488335549539148</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.08037011967511401</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.0361665538538013</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.01394995648646622</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.004708110314182348</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.001412433094254705</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.0003813569354487703</v>
-      </c>
+        <v>16.98076923076923</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>0.006302111920819578</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.03202882452620821</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.08138903382068369</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.1378794450364344</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.1751839941248069</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1780653050317151</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.1508283382016075</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.1095064738055672</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0.06956722758317427</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0.03928412416929229</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.01996512177969077</v>
+      </c>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1558,41 +2195,108 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4.1</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01662938425914923</v>
+        <v>21</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06818047546251182</v>
+        <v>4.79245283018868</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1397699746981492</v>
+        <v>4.870695594904424</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1910189654208039</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.195794439556324</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.1605514404361857</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.1097101509647269</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.06425880270791146</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.03293263638780461</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.01500264546555543</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.006151084640877727</v>
-      </c>
+        <v>15.79245283018868</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="n">
+        <v>0.007757224322108526</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0.03778307833437945</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>0.0920149366025954</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>0.1493922487918904</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>0.1819110420258816</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0.177206662211987</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0.1438532848372736</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0.10009508010992</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0.06094158322037407</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0.03298087788199748</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0.01606398166159259</v>
+      </c>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1601,41 +2305,108 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.9</v>
+        <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>0.05503533924501622</v>
+        <v>23</v>
       </c>
       <c r="D5" t="n">
-        <v>0.159602483810547</v>
+        <v>5.057692307692307</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2314236015252932</v>
+        <v>5.170115567034983</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2237094814744501</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.1621893740689763</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.09406983696000626</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.04546708786400301</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.01883636497222982</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.006828182302433311</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.002200192075228511</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.0006380557018162682</v>
-      </c>
+        <v>18.05769230769231</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="n">
+        <v>0.005782510694012257</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0.02989624855565904</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>0.07728353002677996</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0.1331882605556235</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0.1721496748112352</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0.1780067427203154</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0.1533859052625823</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>0.1132889795088329</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>0.0732146395665155</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0.04205868308418859</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0.02174482521425543</v>
+      </c>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1644,41 +2415,108 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.6</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>0.07428001934180856</v>
+        <v>22</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1931280502887023</v>
+        <v>5.403846153846153</v>
       </c>
       <c r="E6" t="n">
-        <v>0.251066465375313</v>
+        <v>5.578099515742613</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2175909366586045</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.141434108828093</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.07354573659060834</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.03186981918926361</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.01183736141315506</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.003847142459275395</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.001111396710457336</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.0002889631447189074</v>
-      </c>
+        <v>17.40384615384615</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>0.003886828339677544</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.02168111527932997</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.06046970932019514</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.1124353520920257</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.1567938957642197</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.1749223908067583</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.1626224172419531</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0.129589146695176</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.09035764455323243</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.05600265925844766</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.03123884064898455</v>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1687,41 +2525,108 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.5</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2231302832612856</v>
+        <v>17</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3346954248919284</v>
+        <v>4.673076923076923</v>
       </c>
       <c r="E7" t="n">
-        <v>0.2510215686689463</v>
+        <v>4.738966433146786</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1255107843344732</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.04706654412542743</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.01411996323762823</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.003529990809407058</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.000756426602015798</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.0001418299878779621</v>
-      </c>
-      <c r="L7" t="n">
-        <v>2.363833131299369e-05</v>
-      </c>
-      <c r="M7" t="n">
-        <v>3.545749696949053e-06</v>
-      </c>
+        <v>11.67307692307692</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="n">
+        <v>0.008832005957155406</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0.04185457976831192</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0.09917372429774736</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>0.1566603168323928</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.1856019957187125</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>0.1759123255272064</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0.1389404343083703</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0.09406200777060039</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>0.05571958718240842</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>0.02933925036958104</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>0.0139037722675134</v>
+      </c>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1730,40 +2635,107 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.6</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2018967249205256</v>
+        <v>16</v>
       </c>
       <c r="D8" t="n">
-        <v>0.323034759872841</v>
+        <v>4.673076923076923</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2584278078982729</v>
+        <v>4.738966433146786</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1378281642124122</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.05513126568496488</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.01764200501918876</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.00470453467178367</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.00107532221069341</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.0002150644421386821</v>
-      </c>
-      <c r="L8" t="n">
-        <v>3.823367860243238e-05</v>
-      </c>
-      <c r="M8" t="n">
-        <v>6.11738857638918e-06</v>
+        <v>10.67307692307692</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
+      <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="n">
+        <v>0.008832005957155406</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>0.04185457976831192</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>0.09917372429774736</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>0.1566603168323928</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>0.1856019957187125</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>0.1759123255272064</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>0.1389404343083703</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>0.09406200777060039</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>0.05571958718240842</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>0.02933925036958104</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>0.0139037722675134</v>
       </c>
     </row>
   </sheetData>
@@ -1777,7 +2749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1795,51 +2767,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>annual_total_products</t>
+          <t>calendar_year</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7754.2</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>units_per_model_unit</t>
+          <t>annual_total_real_units</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>5689</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>average_daily_demand_in_model_units</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>10.62219178082192</v>
+          <t>annual_weekday_demands_real_units</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[963, 883, 837, 939, 905, 607, 555]</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>max_noise</t>
+          <t>units_per_model_unit</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>max_noise_full_width_model_units</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fit_lambda_to_centered_mean</t>
+        </is>
+      </c>
+      <c r="B7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>max_total_demand_column_K</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D = lower_demand + Z, where Z is truncated Poisson on {0,...,max_noise}; E[D] matches the 2025 weekday mean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>If base demand is 15 and max_noise is 10, support is demand 10 through 20.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kørt flere sens analyser
</commit_message>
<xml_diff>
--- a/weekday_demand_probabilities.xlsx
+++ b/weekday_demand_probabilities.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z8"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,41 +522,6 @@
           <t>demand_17</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>demand_18</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>demand_19</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>demand_20</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>demand_21</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>demand_22</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>demand_23</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>demand_24</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -604,40 +569,19 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>0.1417718949123943</v>
       </c>
       <c r="P2" t="n">
-        <v>0.01041935654618319</v>
+        <v>0.2847392882978802</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.04763277420099123</v>
+        <v>0.2859398273207932</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1088781811058069</v>
+        <v>0.1914302854305798</v>
       </c>
       <c r="S2" t="n">
-        <v>0.165914590248132</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.1896223672476748</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.1733742263743649</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.1320986144163069</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.08627107283950429</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0.04929923592722601</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0.02504163351903341</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0.01144794757477647</v>
+        <v>0.09611870403835249</v>
       </c>
     </row>
     <row r="3">
@@ -683,42 +627,21 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.006302111920819578</v>
+        <v>0.1891687629134388</v>
       </c>
       <c r="O3" t="n">
-        <v>0.03202882452620821</v>
+        <v>0.3206110078465012</v>
       </c>
       <c r="P3" t="n">
-        <v>0.08138903382068369</v>
+        <v>0.2716923681511447</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.1378794450364344</v>
+        <v>0.1534918038890675</v>
       </c>
       <c r="R3" t="n">
-        <v>0.1751839941248069</v>
+        <v>0.06503605719984783</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1780653050317151</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.1508283382016075</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.1095064738055672</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.06956722758317427</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.03928412416929229</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0.01996512177969077</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -762,45 +685,24 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.007757224322108526</v>
+        <v>0.1781918549660359</v>
       </c>
       <c r="N4" t="n">
-        <v>0.03778307833437945</v>
+        <v>0.3134366638260049</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0920149366025954</v>
+        <v>0.2756650752895004</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1493922487918904</v>
+        <v>0.161630173927898</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.1819110420258816</v>
+        <v>0.07107623199056073</v>
       </c>
       <c r="R4" t="n">
-        <v>0.177206662211987</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1438532848372736</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.10009508010992</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.06094158322037407</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.03298087788199748</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.01606398166159259</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -847,42 +749,21 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>0.05451678346039602</v>
       </c>
       <c r="O5" t="n">
-        <v>0.005782510694012257</v>
+        <v>0.171423075865253</v>
       </c>
       <c r="P5" t="n">
-        <v>0.02989624855565904</v>
+        <v>0.2695121490471994</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.07728353002677996</v>
+        <v>0.2824854943144136</v>
       </c>
       <c r="R5" t="n">
-        <v>0.1331882605556235</v>
+        <v>0.2220624973127379</v>
       </c>
       <c r="S5" t="n">
-        <v>0.1721496748112352</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.1780067427203154</v>
-      </c>
-      <c r="U5" t="n">
-        <v>0.1533859052625823</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.1132889795088329</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0.0732146395665155</v>
-      </c>
-      <c r="X5" t="n">
-        <v>0.04205868308418859</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0.02174482521425543</v>
-      </c>
-      <c r="Z5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -929,42 +810,21 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0.003886828339677544</v>
+        <v>0.1228400105152873</v>
       </c>
       <c r="O6" t="n">
-        <v>0.02168111527932997</v>
+        <v>0.2663802161638493</v>
       </c>
       <c r="P6" t="n">
-        <v>0.06046970932019514</v>
+        <v>0.288824542043931</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.1124353520920257</v>
+        <v>0.2087733022825176</v>
       </c>
       <c r="R6" t="n">
-        <v>0.1567938957642197</v>
+        <v>0.1131819289944148</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1749223908067583</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.1626224172419531</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0.129589146695176</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.09035764455323243</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0.05600265925844766</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0.03123884064898455</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -996,57 +856,36 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.008832005957155406</v>
+        <v>0.06572967373390196</v>
       </c>
       <c r="J7" t="n">
-        <v>0.04185457976831192</v>
+        <v>0.1911385221070174</v>
       </c>
       <c r="K7" t="n">
-        <v>0.09917372429774736</v>
+        <v>0.2779105125423082</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1566603168323928</v>
+        <v>0.2693831751971847</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1856019957187125</v>
+        <v>0.1958381164195877</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1759123255272064</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0.1389404343083703</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0.09406200777060039</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.05571958718240842</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>0.02933925036958104</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0139037722675134</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1075,60 +914,39 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0.008832005957155406</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.04185457976831192</v>
+        <v>0.1998809901214293</v>
       </c>
       <c r="J8" t="n">
-        <v>0.09917372429774736</v>
+        <v>0.3270245543310929</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1566603168323928</v>
+        <v>0.2675218365450359</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1856019957187125</v>
+        <v>0.1458971649693938</v>
       </c>
       <c r="M8" t="n">
-        <v>0.1759123255272064</v>
+        <v>0.05967545403304803</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1389404343083703</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>0.09406200777060039</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>0.05571958718240842</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.02933925036958104</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>0.0139037722675134</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1244,40 +1062,40 @@
         <v>18.51923076923077</v>
       </c>
       <c r="E2" t="n">
-        <v>18.51923076923077</v>
+        <v>14.81538461538462</v>
       </c>
       <c r="F2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I2" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="J2" t="n">
-        <v>4.51923076923077</v>
+        <v>1.815384615384616</v>
       </c>
       <c r="K2" t="n">
-        <v>4.57156581501571</v>
+        <v>2.008432549158141</v>
       </c>
       <c r="L2" t="n">
-        <v>4.519230769230769</v>
+        <v>1.815384615384616</v>
       </c>
       <c r="M2" t="n">
-        <v>18.51923076923077</v>
+        <v>14.81538461538462</v>
       </c>
       <c r="N2" t="n">
         <v>18.51923076923077</v>
       </c>
       <c r="O2" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -1296,40 +1114,40 @@
         <v>16.98076923076923</v>
       </c>
       <c r="E3" t="n">
-        <v>16.98076923076923</v>
+        <v>13.58461538461538</v>
       </c>
       <c r="F3" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H3" t="n">
         <v>12</v>
       </c>
       <c r="I3" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J3" t="n">
-        <v>4.98076923076923</v>
+        <v>1.584615384615384</v>
       </c>
       <c r="K3" t="n">
-        <v>5.08223670550791</v>
+        <v>1.69484117202378</v>
       </c>
       <c r="L3" t="n">
-        <v>4.98076923076923</v>
+        <v>1.584615384615384</v>
       </c>
       <c r="M3" t="n">
-        <v>16.98076923076923</v>
+        <v>13.58461538461538</v>
       </c>
       <c r="N3" t="n">
         <v>16.98076923076923</v>
       </c>
       <c r="O3" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1348,40 +1166,40 @@
         <v>15.79245283018868</v>
       </c>
       <c r="E4" t="n">
-        <v>15.79245283018868</v>
+        <v>12.63396226415094</v>
       </c>
       <c r="F4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H4" t="n">
         <v>11</v>
       </c>
       <c r="I4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="J4" t="n">
-        <v>4.79245283018868</v>
+        <v>1.633962264150943</v>
       </c>
       <c r="K4" t="n">
-        <v>4.870695594904424</v>
+        <v>1.758984235759526</v>
       </c>
       <c r="L4" t="n">
-        <v>4.79245283018868</v>
+        <v>1.633962264150943</v>
       </c>
       <c r="M4" t="n">
-        <v>15.79245283018868</v>
+        <v>12.63396226415094</v>
       </c>
       <c r="N4" t="n">
         <v>15.79245283018868</v>
       </c>
       <c r="O4" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -1400,40 +1218,40 @@
         <v>18.05769230769231</v>
       </c>
       <c r="E5" t="n">
-        <v>18.05769230769231</v>
+        <v>14.44615384615384</v>
       </c>
       <c r="F5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I5" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J5" t="n">
-        <v>5.057692307692307</v>
+        <v>2.446153846153845</v>
       </c>
       <c r="K5" t="n">
-        <v>5.170115567034983</v>
+        <v>3.144409207300063</v>
       </c>
       <c r="L5" t="n">
-        <v>5.057692307692307</v>
+        <v>2.446153846153844</v>
       </c>
       <c r="M5" t="n">
-        <v>18.05769230769231</v>
+        <v>14.44615384615384</v>
       </c>
       <c r="N5" t="n">
         <v>18.05769230769231</v>
       </c>
       <c r="O5" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1452,40 +1270,40 @@
         <v>17.40384615384615</v>
       </c>
       <c r="E6" t="n">
-        <v>17.40384615384615</v>
+        <v>13.92307692307692</v>
       </c>
       <c r="F6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H6" t="n">
         <v>12</v>
       </c>
       <c r="I6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J6" t="n">
-        <v>5.403846153846153</v>
+        <v>1.923076923076923</v>
       </c>
       <c r="K6" t="n">
-        <v>5.578099515742613</v>
+        <v>2.168513459470101</v>
       </c>
       <c r="L6" t="n">
-        <v>5.403846153846152</v>
+        <v>1.923076923076923</v>
       </c>
       <c r="M6" t="n">
-        <v>17.40384615384615</v>
+        <v>13.92307692307692</v>
       </c>
       <c r="N6" t="n">
         <v>17.40384615384615</v>
       </c>
       <c r="O6" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1504,40 +1322,40 @@
         <v>11.67307692307692</v>
       </c>
       <c r="E7" t="n">
-        <v>11.67307692307692</v>
+        <v>9.338461538461539</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H7" t="n">
         <v>7</v>
       </c>
       <c r="I7" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J7" t="n">
-        <v>4.673076923076923</v>
+        <v>2.338461538461539</v>
       </c>
       <c r="K7" t="n">
-        <v>4.738966433146786</v>
+        <v>2.907948742919626</v>
       </c>
       <c r="L7" t="n">
-        <v>4.673076923076922</v>
+        <v>2.338461538461539</v>
       </c>
       <c r="M7" t="n">
-        <v>11.67307692307692</v>
+        <v>9.338461538461539</v>
       </c>
       <c r="N7" t="n">
         <v>11.67307692307692</v>
       </c>
       <c r="O7" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -1556,40 +1374,40 @@
         <v>10.67307692307692</v>
       </c>
       <c r="E8" t="n">
-        <v>10.67307692307692</v>
+        <v>8.538461538461538</v>
       </c>
       <c r="F8" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" t="n">
         <v>11</v>
       </c>
-      <c r="G8" t="n">
-        <v>10</v>
-      </c>
-      <c r="H8" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" t="n">
-        <v>16</v>
-      </c>
       <c r="J8" t="n">
-        <v>4.673076923076923</v>
+        <v>1.538461538461538</v>
       </c>
       <c r="K8" t="n">
-        <v>4.738966433146786</v>
+        <v>1.636096329783151</v>
       </c>
       <c r="L8" t="n">
-        <v>4.673076923076922</v>
+        <v>1.538461538461538</v>
       </c>
       <c r="M8" t="n">
-        <v>10.67307692307692</v>
+        <v>8.538461538461538</v>
       </c>
       <c r="N8" t="n">
         <v>10.67307692307692</v>
       </c>
       <c r="O8" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="P8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1603,7 +1421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT8"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1639,332 +1457,102 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_0_demand_14</t>
+          <t>P_offset_0_demand_13</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_1_demand_15</t>
+          <t>P_offset_1_demand_14</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_2_demand_16</t>
+          <t>P_offset_2_demand_15</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_3_demand_17</t>
+          <t>P_offset_3_demand_16</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_4_demand_18</t>
+          <t>P_offset_4_demand_17</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_5_demand_19</t>
+          <t>P_offset_0_demand_12</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_6_demand_20</t>
+          <t>P_offset_1_demand_13</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_7_demand_21</t>
+          <t>P_offset_2_demand_14</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_8_demand_22</t>
+          <t>P_offset_3_demand_15</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_9_demand_23</t>
+          <t>P_offset_4_demand_16</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_10_demand_24</t>
+          <t>P_offset_0_demand_11</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_0_demand_12</t>
+          <t>P_offset_1_demand_12</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_1_demand_13</t>
+          <t>P_offset_2_demand_13</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_2_demand_14</t>
+          <t>P_offset_3_demand_14</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_3_demand_15</t>
+          <t>P_offset_4_demand_15</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_4_demand_16</t>
+          <t>P_offset_0_demand_7</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_5_demand_17</t>
+          <t>P_offset_1_demand_8</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_6_demand_18</t>
+          <t>P_offset_2_demand_9</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_7_demand_19</t>
+          <t>P_offset_3_demand_10</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>P_offset_8_demand_20</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_9_demand_21</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_10_demand_22</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_0_demand_11</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_1_demand_12</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_2_demand_13</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_3_demand_14</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_4_demand_15</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_5_demand_16</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_6_demand_17</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_7_demand_18</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_8_demand_19</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_9_demand_20</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_10_demand_21</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_0_demand_13</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_1_demand_14</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_2_demand_15</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_3_demand_16</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_4_demand_17</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_5_demand_18</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_6_demand_19</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_7_demand_20</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_8_demand_21</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_9_demand_22</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_10_demand_23</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_0_demand_7</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_1_demand_8</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_2_demand_9</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_3_demand_10</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
           <t>P_offset_4_demand_11</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_5_demand_12</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_6_demand_13</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_7_demand_14</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_8_demand_15</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_9_demand_16</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_10_demand_17</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_0_demand_6</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_1_demand_7</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_2_demand_8</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_3_demand_9</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_4_demand_10</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_5_demand_11</t>
-        </is>
-      </c>
-      <c r="BP1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_6_demand_12</t>
-        </is>
-      </c>
-      <c r="BQ1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_7_demand_13</t>
-        </is>
-      </c>
-      <c r="BR1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_8_demand_14</t>
-        </is>
-      </c>
-      <c r="BS1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_9_demand_15</t>
-        </is>
-      </c>
-      <c r="BT1" s="1" t="inlineStr">
-        <is>
-          <t>P_offset_10_demand_16</t>
         </is>
       </c>
     </row>
@@ -1975,53 +1563,41 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>4.51923076923077</v>
+        <v>1.815384615384616</v>
       </c>
       <c r="E2" t="n">
-        <v>4.57156581501571</v>
+        <v>2.008432549158141</v>
       </c>
       <c r="F2" t="n">
-        <v>18.51923076923077</v>
+        <v>14.81538461538462</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01041935654618319</v>
+        <v>0.1417718949123943</v>
       </c>
       <c r="H2" t="n">
-        <v>0.04763277420099123</v>
+        <v>0.2847392882978802</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1088781811058069</v>
+        <v>0.2859398273207932</v>
       </c>
       <c r="J2" t="n">
-        <v>0.165914590248132</v>
+        <v>0.1914302854305798</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1896223672476748</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.1733742263743649</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.1320986144163069</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.08627107283950429</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.04929923592722601</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.02504163351903341</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.01144794757477647</v>
-      </c>
+        <v>0.09611870403835249</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
@@ -2031,52 +1607,6 @@
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2088,105 +1618,47 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>4.98076923076923</v>
+        <v>1.584615384615384</v>
       </c>
       <c r="E3" t="n">
-        <v>5.08223670550791</v>
+        <v>1.69484117202378</v>
       </c>
       <c r="F3" t="n">
-        <v>16.98076923076923</v>
+        <v>13.58461538461538</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0.1891687629134388</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.3206110078465012</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.2716923681511447</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.1534918038890675</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.06503605719984783</v>
+      </c>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="n">
-        <v>0.006302111920819578</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.03202882452620821</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.08138903382068369</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.1378794450364344</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.1751839941248069</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.1780653050317151</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0.1508283382016075</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0.1095064738055672</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0.06956722758317427</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0.03928412416929229</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>0.01996512177969077</v>
-      </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
-      <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
-      <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="inlineStr"/>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr"/>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2198,16 +1670,16 @@
         <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D4" t="n">
-        <v>4.79245283018868</v>
+        <v>1.633962264150943</v>
       </c>
       <c r="E4" t="n">
-        <v>4.870695594904424</v>
+        <v>1.758984235759526</v>
       </c>
       <c r="F4" t="n">
-        <v>15.79245283018868</v>
+        <v>12.63396226415094</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -2219,84 +1691,26 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="Q4" t="n">
+        <v>0.1781918549660359</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.3134366638260049</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.2756650752895004</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.161630173927898</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.07107623199056073</v>
+      </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="n">
-        <v>0.007757224322108526</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.03778307833437945</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>0.0920149366025954</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0.1493922487918904</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>0.1819110420258816</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0.177206662211987</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>0.1438532848372736</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>0.10009508010992</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0.06094158322037407</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0.03298087788199748</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0.01606398166159259</v>
-      </c>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
-      <c r="BG4" t="inlineStr"/>
-      <c r="BH4" t="inlineStr"/>
-      <c r="BI4" t="inlineStr"/>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="inlineStr"/>
-      <c r="BM4" t="inlineStr"/>
-      <c r="BN4" t="inlineStr"/>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="inlineStr"/>
-      <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2305,30 +1719,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>5.057692307692307</v>
+        <v>2.446153846153845</v>
       </c>
       <c r="E5" t="n">
-        <v>5.170115567034983</v>
+        <v>3.144409207300063</v>
       </c>
       <c r="F5" t="n">
-        <v>18.05769230769231</v>
+        <v>14.44615384615384</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0.05451678346039602</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.171423075865253</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.2695121490471994</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.2824854943144136</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.2220624973127379</v>
+      </c>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
@@ -2339,74 +1763,6 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="n">
-        <v>0.005782510694012257</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>0.02989624855565904</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>0.07728353002677996</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0.1331882605556235</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>0.1721496748112352</v>
-      </c>
-      <c r="AS5" t="n">
-        <v>0.1780067427203154</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>0.1533859052625823</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>0.1132889795088329</v>
-      </c>
-      <c r="AV5" t="n">
-        <v>0.0732146395665155</v>
-      </c>
-      <c r="AW5" t="n">
-        <v>0.04205868308418859</v>
-      </c>
-      <c r="AX5" t="n">
-        <v>0.02174482521425543</v>
-      </c>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
-      <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
-      <c r="BF5" t="inlineStr"/>
-      <c r="BG5" t="inlineStr"/>
-      <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="inlineStr"/>
-      <c r="BJ5" t="inlineStr"/>
-      <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="inlineStr"/>
-      <c r="BM5" t="inlineStr"/>
-      <c r="BN5" t="inlineStr"/>
-      <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr"/>
-      <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="inlineStr"/>
-      <c r="BS5" t="inlineStr"/>
-      <c r="BT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2418,105 +1774,47 @@
         <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>5.403846153846153</v>
+        <v>1.923076923076923</v>
       </c>
       <c r="E6" t="n">
-        <v>5.578099515742613</v>
+        <v>2.168513459470101</v>
       </c>
       <c r="F6" t="n">
-        <v>17.40384615384615</v>
+        <v>13.92307692307692</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0.1228400105152873</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.2663802161638493</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.288824542043931</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.2087733022825176</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.1131819289944148</v>
+      </c>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="n">
-        <v>0.003886828339677544</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.02168111527932997</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.06046970932019514</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0.1124353520920257</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.1567938957642197</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0.1749223908067583</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0.1626224172419531</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>0.129589146695176</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0.09035764455323243</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0.05600265925844766</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0.03123884064898455</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
-      <c r="BF6" t="inlineStr"/>
-      <c r="BG6" t="inlineStr"/>
-      <c r="BH6" t="inlineStr"/>
-      <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
-      <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
-      <c r="BM6" t="inlineStr"/>
-      <c r="BN6" t="inlineStr"/>
-      <c r="BO6" t="inlineStr"/>
-      <c r="BP6" t="inlineStr"/>
-      <c r="BQ6" t="inlineStr"/>
-      <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="inlineStr"/>
-      <c r="BT6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2528,16 +1826,16 @@
         <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>4.673076923076923</v>
+        <v>2.338461538461539</v>
       </c>
       <c r="E7" t="n">
-        <v>4.738966433146786</v>
+        <v>2.907948742919626</v>
       </c>
       <c r="F7" t="n">
-        <v>11.67307692307692</v>
+        <v>9.338461538461539</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -2554,79 +1852,21 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="n">
-        <v>0.008832005957155406</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>0.04185457976831192</v>
-      </c>
-      <c r="BA7" t="n">
-        <v>0.09917372429774736</v>
-      </c>
-      <c r="BB7" t="n">
-        <v>0.1566603168323928</v>
-      </c>
-      <c r="BC7" t="n">
-        <v>0.1856019957187125</v>
-      </c>
-      <c r="BD7" t="n">
-        <v>0.1759123255272064</v>
-      </c>
-      <c r="BE7" t="n">
-        <v>0.1389404343083703</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>0.09406200777060039</v>
-      </c>
-      <c r="BG7" t="n">
-        <v>0.05571958718240842</v>
-      </c>
-      <c r="BH7" t="n">
-        <v>0.02933925036958104</v>
-      </c>
-      <c r="BI7" t="n">
-        <v>0.0139037722675134</v>
-      </c>
-      <c r="BJ7" t="inlineStr"/>
-      <c r="BK7" t="inlineStr"/>
-      <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
-      <c r="BN7" t="inlineStr"/>
-      <c r="BO7" t="inlineStr"/>
-      <c r="BP7" t="inlineStr"/>
-      <c r="BQ7" t="inlineStr"/>
-      <c r="BR7" t="inlineStr"/>
-      <c r="BS7" t="inlineStr"/>
-      <c r="BT7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>0.06572967373390196</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.1911385221070174</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0.2779105125423082</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0.2693831751971847</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0.1958381164195877</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2635,19 +1875,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D8" t="n">
-        <v>4.673076923076923</v>
+        <v>1.538461538461538</v>
       </c>
       <c r="E8" t="n">
-        <v>4.738966433146786</v>
+        <v>1.636096329783151</v>
       </c>
       <c r="F8" t="n">
-        <v>10.67307692307692</v>
+        <v>8.538461538461538</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -2664,78 +1904,20 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
-      <c r="BF8" t="inlineStr"/>
-      <c r="BG8" t="inlineStr"/>
-      <c r="BH8" t="inlineStr"/>
-      <c r="BI8" t="inlineStr"/>
-      <c r="BJ8" t="n">
-        <v>0.008832005957155406</v>
-      </c>
-      <c r="BK8" t="n">
-        <v>0.04185457976831192</v>
-      </c>
-      <c r="BL8" t="n">
-        <v>0.09917372429774736</v>
-      </c>
-      <c r="BM8" t="n">
-        <v>0.1566603168323928</v>
-      </c>
-      <c r="BN8" t="n">
-        <v>0.1856019957187125</v>
-      </c>
-      <c r="BO8" t="n">
-        <v>0.1759123255272064</v>
-      </c>
-      <c r="BP8" t="n">
-        <v>0.1389404343083703</v>
-      </c>
-      <c r="BQ8" t="n">
-        <v>0.09406200777060039</v>
-      </c>
-      <c r="BR8" t="n">
-        <v>0.05571958718240842</v>
-      </c>
-      <c r="BS8" t="n">
-        <v>0.02933925036958104</v>
-      </c>
-      <c r="BT8" t="n">
-        <v>0.0139037722675134</v>
+      <c r="V8" t="n">
+        <v>0.1998809901214293</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.3270245543310929</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0.2675218365450359</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0.1458971649693938</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0.05967545403304803</v>
       </c>
     </row>
   </sheetData>
@@ -2803,7 +1985,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="6">
@@ -2813,7 +1995,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -2833,7 +2015,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">

</xml_diff>